<commit_message>
Tieup Program change window
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testData/input_UserRights.xlsx
+++ b/testData/input_UserRights.xlsx
@@ -476,7 +476,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Varsha Jha</t>
+          <t>Shivali Gupta</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -491,17 +491,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Nidhi Chaturvedi</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Transport</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Raise_Support_Request</t>
         </is>

</xml_diff>